<commit_message>
upd data sheet, uploaded set 2 of images for week 02 and the week 01 1st image set, will explain soon. Added some explination text
</commit_message>
<xml_diff>
--- a/Data Record.xlsx
+++ b/Data Record.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\GitHub\Dear-Data-100\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3D5B774-DBF8-40B6-9E07-FDFFC6BA60A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B9B0A31-3F45-4B65-9756-0B5AC6119BFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3300" yWindow="1590" windowWidth="22065" windowHeight="12345" xr2:uid="{E1609FB1-39BB-4B4B-BB31-177E3FF80247}"/>
+    <workbookView xWindow="2928" yWindow="2928" windowWidth="17280" windowHeight="9984" xr2:uid="{E1609FB1-39BB-4B4B-BB31-177E3FF80247}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -249,7 +249,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -259,9 +259,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
@@ -280,6 +277,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>356169</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>5035</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0A23E8C2-4B8D-03E8-349C-1C7FFCDDA879}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6079901" y="1126901"/>
+          <a:ext cx="9457240" cy="5467824"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -600,13 +646,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{808E46E3-39F5-40CF-B2AC-C00C723DC56C}">
   <dimension ref="A1:AB40"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="5.42578125" customWidth="1"/>
-    <col min="2" max="28" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="5.41796875" customWidth="1"/>
+    <col min="2" max="28" width="15.68359375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
         <v>8</v>
@@ -690,7 +736,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
@@ -722,16 +768,16 @@
       <c r="AA2" s="3"/>
       <c r="AB2" s="3"/>
     </row>
-    <row r="3" spans="1:28" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" ht="60" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7" t="s">
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="5" t="s">
         <v>38</v>
       </c>
       <c r="F3" s="5" t="s">
@@ -761,7 +807,7 @@
       <c r="V3" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="W3" s="7" t="s">
+      <c r="W3" s="5" t="s">
         <v>41</v>
       </c>
       <c r="X3" s="5" t="s">
@@ -774,7 +820,7 @@
       <c r="AA3" s="5"/>
       <c r="AB3" s="5"/>
     </row>
-    <row r="4" spans="1:28" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" ht="60" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
@@ -806,7 +852,7 @@
       <c r="AA4" s="5"/>
       <c r="AB4" s="5"/>
     </row>
-    <row r="5" spans="1:28" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" ht="59.25" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
@@ -838,7 +884,7 @@
       <c r="AA5" s="5"/>
       <c r="AB5" s="5"/>
     </row>
-    <row r="6" spans="1:28" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28" ht="60" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="2" t="s">
         <v>1</v>
       </c>
@@ -870,7 +916,7 @@
       <c r="AA6" s="5"/>
       <c r="AB6" s="5"/>
     </row>
-    <row r="7" spans="1:28" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:28" ht="60" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="2" t="s">
         <v>3</v>
       </c>
@@ -902,7 +948,7 @@
       <c r="AA7" s="5"/>
       <c r="AB7" s="5"/>
     </row>
-    <row r="8" spans="1:28" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" ht="59.25" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="2" t="s">
         <v>4</v>
       </c>
@@ -934,7 +980,7 @@
       <c r="AA8" s="5"/>
       <c r="AB8" s="5"/>
     </row>
-    <row r="9" spans="1:28" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:28" ht="60" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="2" t="s">
         <v>4</v>
       </c>
@@ -966,7 +1012,7 @@
       <c r="AA9" s="5"/>
       <c r="AB9" s="5"/>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="3" t="s">
         <v>6</v>
       </c>
@@ -998,7 +1044,7 @@
       <c r="AA10" s="3"/>
       <c r="AB10" s="3"/>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="2" t="s">
         <v>0</v>
       </c>
@@ -1030,7 +1076,7 @@
       <c r="AA11" s="4"/>
       <c r="AB11" s="4"/>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="2" t="s">
         <v>1</v>
       </c>
@@ -1062,7 +1108,7 @@
       <c r="AA12" s="4"/>
       <c r="AB12" s="4"/>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="2" t="s">
         <v>2</v>
       </c>
@@ -1094,7 +1140,7 @@
       <c r="AA13" s="4"/>
       <c r="AB13" s="4"/>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="2" t="s">
         <v>1</v>
       </c>
@@ -1126,7 +1172,7 @@
       <c r="AA14" s="4"/>
       <c r="AB14" s="4"/>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="2" t="s">
         <v>3</v>
       </c>
@@ -1158,7 +1204,7 @@
       <c r="AA15" s="4"/>
       <c r="AB15" s="4"/>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="2" t="s">
         <v>4</v>
       </c>
@@ -1190,7 +1236,7 @@
       <c r="AA16" s="4"/>
       <c r="AB16" s="4"/>
     </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="2" t="s">
         <v>4</v>
       </c>
@@ -1222,7 +1268,7 @@
       <c r="AA17" s="4"/>
       <c r="AB17" s="4"/>
     </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="3" t="s">
         <v>7</v>
       </c>
@@ -1254,7 +1300,7 @@
       <c r="AA18" s="3"/>
       <c r="AB18" s="3"/>
     </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="2" t="s">
         <v>0</v>
       </c>
@@ -1286,7 +1332,7 @@
       <c r="AA19" s="4"/>
       <c r="AB19" s="4"/>
     </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="2" t="s">
         <v>1</v>
       </c>
@@ -1318,7 +1364,7 @@
       <c r="AA20" s="4"/>
       <c r="AB20" s="4"/>
     </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="2" t="s">
         <v>2</v>
       </c>
@@ -1350,7 +1396,7 @@
       <c r="AA21" s="4"/>
       <c r="AB21" s="4"/>
     </row>
-    <row r="22" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="2" t="s">
         <v>1</v>
       </c>
@@ -1382,7 +1428,7 @@
       <c r="AA22" s="4"/>
       <c r="AB22" s="4"/>
     </row>
-    <row r="23" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="2" t="s">
         <v>3</v>
       </c>
@@ -1414,7 +1460,7 @@
       <c r="AA23" s="4"/>
       <c r="AB23" s="4"/>
     </row>
-    <row r="24" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="2" t="s">
         <v>4</v>
       </c>
@@ -1446,7 +1492,7 @@
       <c r="AA24" s="4"/>
       <c r="AB24" s="4"/>
     </row>
-    <row r="25" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="2" t="s">
         <v>4</v>
       </c>
@@ -1478,63 +1524,64 @@
       <c r="AA25" s="4"/>
       <c r="AB25" s="4"/>
     </row>
-    <row r="26" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="1"/>
     </row>
-    <row r="27" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="1"/>
     </row>
-    <row r="28" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="1"/>
     </row>
-    <row r="29" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="1"/>
     </row>
-    <row r="30" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="1"/>
     </row>
-    <row r="31" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="1"/>
     </row>
-    <row r="32" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="1"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="1"/>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="1"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="1"/>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="1"/>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="1"/>
     </row>
-    <row r="38" spans="1:13" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:13" ht="58.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="1"/>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B40" s="8" t="s">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.55000000000000004">
+      <c r="B40" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="C40" s="8"/>
-      <c r="D40" s="8"/>
-      <c r="E40" s="8"/>
-      <c r="F40" s="8"/>
-      <c r="G40" s="8"/>
-      <c r="H40" s="8"/>
-      <c r="I40" s="8"/>
-      <c r="J40" s="8"/>
-      <c r="K40" s="8"/>
-      <c r="L40" s="8"/>
-      <c r="M40" s="8"/>
+      <c r="C40" s="7"/>
+      <c r="D40" s="7"/>
+      <c r="E40" s="7"/>
+      <c r="F40" s="7"/>
+      <c r="G40" s="7"/>
+      <c r="H40" s="7"/>
+      <c r="I40" s="7"/>
+      <c r="J40" s="7"/>
+      <c r="K40" s="7"/>
+      <c r="L40" s="7"/>
+      <c r="M40" s="7"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>